<commit_message>
docs: finalize phase 1-3 report and complete team workbook for member 1
</commit_message>
<xml_diff>
--- a/SE_Lab_QT2_Assignment1_Team_Workbook_Template.xlsx
+++ b/SE_Lab_QT2_Assignment1_Team_Workbook_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CNPM\assignment1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AABA9DB9-383F-4190-BBA4-EFACADEA69D1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C4A934F-094B-4319-B75F-3BB016E71D04}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" tabRatio="769" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" tabRatio="769" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="485">
   <si>
     <t>SE Lab Assignment 1 Team Workbook</t>
   </si>
@@ -1350,6 +1350,147 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>29/10</t>
+  </si>
+  <si>
+    <t>main</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>[Commit 4f39f48] Completed Phase 1-3 Requirements (FR/NFR/DR), Clarification Q&amp;A, and UC1 Specification.</t>
+  </si>
+  <si>
+    <t>https://github.com/seuquay56/SmartTicketingSystem_TVM</t>
+  </si>
+  <si>
+    <t>DR1</t>
+  </si>
+  <si>
+    <t>The system shall generate printed ticket barcodes compliant with public transport encoding rules.</t>
+  </si>
+  <si>
+    <t>Domain</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>ISO/IEC 18004 QR Code Standard</t>
+  </si>
+  <si>
+    <t>Barcode scanner validation</t>
+  </si>
+  <si>
+    <t>DR2</t>
+  </si>
+  <si>
+    <t>The system shall process credit card payments in compliance with payment industry data security guidelines.</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>PCI-DSS &amp; EMV Payment Standard</t>
+  </si>
+  <si>
+    <t>Security compliance audit</t>
+  </si>
+  <si>
+    <t>Word</t>
+  </si>
+  <si>
+    <t>Excel</t>
+  </si>
+  <si>
+    <t>Section 2.1</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Section 2.2</t>
+  </si>
+  <si>
+    <t>Section 3.1.3</t>
+  </si>
+  <si>
+    <t>Git</t>
+  </si>
+  <si>
+    <t>[https://github.com/seuquay56/SmartTicketingSystem_TVM](https://github.com/seuquay56/SmartTicketingSystem_TVM)</t>
+  </si>
+  <si>
+    <t>Gemini / ChatGPT</t>
+  </si>
+  <si>
+    <t>Section 5.2.2</t>
+  </si>
+  <si>
+    <t>Gemini</t>
+  </si>
+  <si>
+    <t>Soạn giúp tôi 3 câu hỏi Clarification Q&amp;A cho hệ thống TVM tập trung vào lỗi thanh toán và kẹt giấy.</t>
+  </si>
+  <si>
+    <t>Gợi ý các tình huống biên và giải pháp xử lý lỗi phần cứng (kẹt giấy, hết giấy, timeout).</t>
+  </si>
+  <si>
+    <t>Đối chiếu với thực tế vận hành máy kiosk tự phục vụ và các kịch bản hoàn tiền tự động.</t>
+  </si>
+  <si>
+    <t>Requirements Spec</t>
+  </si>
+  <si>
+    <t>Chuyển đổi các câu Q&amp;A thành bảng FR1-FR7, NFR1-NFR4 có chỉ số đo lường cụ thể cho NFR.</t>
+  </si>
+  <si>
+    <t>Tạo mẫu bảng chuẩn IEEE 830 và đặt metric thời gian phản hồi (&lt;1.0s, &lt;2.0s).</t>
+  </si>
+  <si>
+    <t>Use Case UC01 Spec</t>
+  </si>
+  <si>
+    <t>Viết đặc tả Use Case UC01 Buy a Ticket gồm Main Flow 10 bước, Alternate Flow và Exception Flow.</t>
+  </si>
+  <si>
+    <t>Sinh luồng sự kiện chi tiết và phân định rõ hành vi của Passenger, Gateway, Printer.</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>Git Troubleshooting</t>
+  </si>
+  <si>
+    <t>Sửa lỗi git rebase lock và dọn dẹp các file rác Office ~$*.docx khỏi repository.</t>
+  </si>
+  <si>
+    <t>Cung cấp chuỗi lệnh git rebase --abort và git rm -f --cached '~$*'.</t>
+  </si>
+  <si>
+    <t>28/10</t>
+  </si>
+  <si>
+    <t>Formed team, setup GitHub repository, completed Clarification Q&amp;A (Q01-Q03).</t>
+  </si>
+  <si>
+    <t>Commit f86f2bc</t>
+  </si>
+  <si>
+    <t>None. Project setup and GitHub integration went smoothly.</t>
+  </si>
+  <si>
+    <t>Resolved Git rebase conflicts and cleaned temporary Office lock files (~$*) from repository.</t>
+  </si>
+  <si>
+    <t>Completed FR1-FR7, NFR1-NFR4, DR1-DR2, and UC01 detailed specification.</t>
+  </si>
+  <si>
+    <t>Commit 4f39f48</t>
   </si>
 </sst>
 </file>
@@ -1360,7 +1501,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="\+0.0;\-0.0;0.0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1427,6 +1568,14 @@
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1497,10 +1646,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1602,10 +1752,28 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1617,8 +1785,12 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
@@ -2043,12 +2215,12 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
     </row>
     <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
@@ -2056,36 +2228,36 @@
       </c>
     </row>
     <row r="8" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="37"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
+      <c r="B8" s="42"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
     </row>
     <row r="9" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
     </row>
     <row r="10" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
+      <c r="B10" s="42"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
     </row>
     <row r="11" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="37" t="s">
+      <c r="A11" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
     </row>
     <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
@@ -2361,10 +2533,18 @@
       <c r="B5" s="4" t="s">
         <v>291</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
+      <c r="C5" s="41" t="s">
+        <v>479</v>
+      </c>
+      <c r="D5" s="41" t="s">
+        <v>480</v>
+      </c>
+      <c r="E5" s="41" t="s">
+        <v>481</v>
+      </c>
+      <c r="F5" s="41" t="s">
+        <v>457</v>
+      </c>
       <c r="G5" s="6"/>
       <c r="H5" s="21"/>
     </row>
@@ -2375,10 +2555,18 @@
       <c r="B6" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
+      <c r="C6" s="41" t="s">
+        <v>483</v>
+      </c>
+      <c r="D6" s="41" t="s">
+        <v>484</v>
+      </c>
+      <c r="E6" s="41" t="s">
+        <v>482</v>
+      </c>
+      <c r="F6" s="41" t="s">
+        <v>457</v>
+      </c>
       <c r="G6" s="6"/>
       <c r="H6" s="21"/>
     </row>
@@ -2391,7 +2579,7 @@
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
+      <c r="E7" s="41"/>
       <c r="F7" s="4"/>
       <c r="G7" s="6"/>
       <c r="H7" s="21"/>
@@ -2454,7 +2642,7 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="F5:F10" xr:uid="{00000000-0002-0000-0900-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="F7:F10" xr:uid="{00000000-0002-0000-0900-000000000000}">
       <formula1>"On track,Behind,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2464,7 +2652,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2820,11 +3008,11 @@
       <c r="A4" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="40">
+      <c r="B4" s="46">
         <f>IF(Team!B4="","",Team!B4)</f>
         <v>14</v>
       </c>
-      <c r="C4" s="40"/>
+      <c r="C4" s="46"/>
     </row>
     <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
@@ -3055,23 +3243,23 @@
       <c r="A25" s="9" t="s">
         <v>349</v>
       </c>
-      <c r="B25" s="38"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="38"/>
+      <c r="B25" s="43"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="43"/>
+      <c r="F25" s="43"/>
+      <c r="G25" s="43"/>
     </row>
     <row r="26" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>290</v>
       </c>
-      <c r="B26" s="41"/>
-      <c r="C26" s="41"/>
-      <c r="D26" s="41"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
-      <c r="G26" s="41"/>
+      <c r="B26" s="47"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="47"/>
+      <c r="E26" s="47"/>
+      <c r="F26" s="47"/>
+      <c r="G26" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3125,18 +3313,20 @@
       <c r="A4" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="38">
+      <c r="B4" s="43">
         <v>14</v>
       </c>
-      <c r="C4" s="38"/>
+      <c r="C4" s="43"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
+      <c r="B5" s="44" t="s">
+        <v>442</v>
+      </c>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
@@ -3150,12 +3340,12 @@
       <c r="A7" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="39" t="str">
+      <c r="B7" s="45" t="str">
         <f>IF(AND(B6&gt;=3,B6&lt;=5),"OK","Group must have 3 to 5 students")</f>
         <v>OK</v>
       </c>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="45"/>
     </row>
     <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
@@ -3201,13 +3391,13 @@
       <c r="E11" s="12">
         <v>0.3</v>
       </c>
-      <c r="F11" s="10">
+      <c r="F11" s="38">
         <f>IF(C11="","",SUMIF('Commit Log'!$C$5:$C$64,C11,'Commit Log'!$E$5:$E$64))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="10" t="str">
         <f>IF(C11="","",IF(AND(ISNUMBER(F11),F11&gt;0),"OK","No commits yet"))</f>
-        <v>No commits yet</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
@@ -3344,8 +3534,11 @@
       <formula2>1</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{CCA07C0A-6BC5-4E7C-A489-F8490F41DD45}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3710,33 +3903,63 @@
       <c r="J14" s="6"/>
     </row>
     <row r="15" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="str">
-        <f>IF(C15="","",C15&amp;COUNTIF($C$5:C15,C15))</f>
-        <v/>
-      </c>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
+      <c r="A15" s="16" t="s">
+        <v>443</v>
+      </c>
+      <c r="B15" s="39" t="s">
+        <v>444</v>
+      </c>
+      <c r="C15" s="39" t="s">
+        <v>445</v>
+      </c>
+      <c r="D15" s="39" t="s">
+        <v>446</v>
+      </c>
+      <c r="E15" s="39" t="s">
+        <v>447</v>
+      </c>
+      <c r="F15" s="39" t="s">
+        <v>448</v>
+      </c>
+      <c r="G15" s="39" t="s">
+        <v>374</v>
+      </c>
+      <c r="H15" s="39" t="s">
+        <v>390</v>
+      </c>
+      <c r="I15" s="39" t="s">
+        <v>376</v>
+      </c>
       <c r="J15" s="6"/>
     </row>
     <row r="16" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="str">
-        <f>IF(C16="","",C16&amp;COUNTIF($C$5:C16,C16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
+      <c r="A16" s="16" t="s">
+        <v>449</v>
+      </c>
+      <c r="B16" s="39" t="s">
+        <v>450</v>
+      </c>
+      <c r="C16" s="39" t="s">
+        <v>445</v>
+      </c>
+      <c r="D16" s="39" t="s">
+        <v>451</v>
+      </c>
+      <c r="E16" s="39" t="s">
+        <v>452</v>
+      </c>
+      <c r="F16" s="39" t="s">
+        <v>453</v>
+      </c>
+      <c r="G16" s="39" t="s">
+        <v>374</v>
+      </c>
+      <c r="H16" s="39" t="s">
+        <v>386</v>
+      </c>
+      <c r="I16" s="39" t="s">
+        <v>376</v>
+      </c>
       <c r="J16" s="6"/>
     </row>
     <row r="17" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4378,27 +4601,27 @@
       <formula>C62&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E15:E54">
+  <conditionalFormatting sqref="E17:E54">
     <cfRule type="expression" dxfId="5" priority="2">
-      <formula>AND($C15="NFR",$E15="",$B15&lt;&gt;"")</formula>
+      <formula>AND($C17="NFR",$E17="",$B17&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose a value from the list." sqref="C15:C54" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose a value from the list." sqref="C17:C54" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"FR,NFR,DR"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose a value from the list." sqref="D15:D54" xr:uid="{00000000-0002-0000-0300-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose a value from the list." sqref="D17:D54" xr:uid="{00000000-0002-0000-0300-000001000000}">
       <formula1>"Reliability,Response time,Availability,Security,Usability,Capacity,Maintainability,Other"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose a value from the list." sqref="G15:G54" xr:uid="{00000000-0002-0000-0300-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose a value from the list." sqref="G17:G54" xr:uid="{00000000-0002-0000-0300-000002000000}">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4975,25 +5198,25 @@
       <c r="A5" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="39" t="s">
         <v>422</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="39" t="s">
         <v>423</v>
       </c>
-      <c r="D5" s="35" t="s">
+      <c r="D5" s="39" t="s">
         <v>424</v>
       </c>
-      <c r="E5" s="35" t="s">
+      <c r="E5" s="39" t="s">
         <v>436</v>
       </c>
-      <c r="F5" s="35" t="s">
+      <c r="F5" s="39" t="s">
         <v>437</v>
       </c>
-      <c r="G5" s="35" t="s">
+      <c r="G5" s="39" t="s">
         <v>437</v>
       </c>
-      <c r="H5" s="35" t="s">
+      <c r="H5" s="39" t="s">
         <v>414</v>
       </c>
       <c r="I5" s="6"/>
@@ -5002,25 +5225,25 @@
       <c r="A6" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="39" t="s">
         <v>425</v>
       </c>
-      <c r="C6" s="35" t="s">
+      <c r="C6" s="39" t="s">
         <v>423</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="39" t="s">
         <v>426</v>
       </c>
-      <c r="E6" s="35" t="s">
+      <c r="E6" s="39" t="s">
         <v>427</v>
       </c>
-      <c r="F6" s="35" t="s">
+      <c r="F6" s="39" t="s">
         <v>437</v>
       </c>
-      <c r="G6" s="35" t="s">
+      <c r="G6" s="39" t="s">
         <v>437</v>
       </c>
-      <c r="H6" s="35" t="s">
+      <c r="H6" s="39" t="s">
         <v>414</v>
       </c>
       <c r="I6" s="6"/>
@@ -5029,25 +5252,25 @@
       <c r="A7" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="39" t="s">
         <v>428</v>
       </c>
-      <c r="C7" s="35" t="s">
+      <c r="C7" s="39" t="s">
         <v>423</v>
       </c>
-      <c r="D7" s="35" t="s">
+      <c r="D7" s="39" t="s">
         <v>429</v>
       </c>
-      <c r="E7" s="35" t="s">
+      <c r="E7" s="39" t="s">
         <v>430</v>
       </c>
-      <c r="F7" s="35" t="s">
+      <c r="F7" s="39" t="s">
         <v>437</v>
       </c>
-      <c r="G7" s="35" t="s">
+      <c r="G7" s="39" t="s">
         <v>437</v>
       </c>
-      <c r="H7" s="35" t="s">
+      <c r="H7" s="39" t="s">
         <v>414</v>
       </c>
       <c r="I7" s="6"/>
@@ -5056,25 +5279,25 @@
       <c r="A8" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="B8" s="35" t="s">
+      <c r="B8" s="39" t="s">
         <v>431</v>
       </c>
-      <c r="C8" s="35" t="s">
+      <c r="C8" s="39" t="s">
         <v>432</v>
       </c>
-      <c r="D8" s="35" t="s">
+      <c r="D8" s="39" t="s">
         <v>433</v>
       </c>
-      <c r="E8" s="35" t="s">
+      <c r="E8" s="39" t="s">
         <v>388</v>
       </c>
-      <c r="F8" s="35" t="s">
+      <c r="F8" s="39" t="s">
         <v>437</v>
       </c>
-      <c r="G8" s="35" t="s">
+      <c r="G8" s="39" t="s">
         <v>437</v>
       </c>
-      <c r="H8" s="35" t="s">
+      <c r="H8" s="39" t="s">
         <v>414</v>
       </c>
       <c r="I8" s="6"/>
@@ -5083,25 +5306,25 @@
       <c r="A9" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="39" t="s">
         <v>434</v>
       </c>
-      <c r="C9" s="35" t="s">
+      <c r="C9" s="39" t="s">
         <v>423</v>
       </c>
-      <c r="D9" s="35" t="s">
+      <c r="D9" s="39" t="s">
         <v>435</v>
       </c>
-      <c r="E9" s="35" t="s">
+      <c r="E9" s="39" t="s">
         <v>391</v>
       </c>
-      <c r="F9" s="35" t="s">
+      <c r="F9" s="39" t="s">
         <v>437</v>
       </c>
-      <c r="G9" s="35" t="s">
+      <c r="G9" s="39" t="s">
         <v>437</v>
       </c>
-      <c r="H9" s="35" t="s">
+      <c r="H9" s="39" t="s">
         <v>414</v>
       </c>
       <c r="I9" s="6"/>
@@ -5281,13 +5504,21 @@
       <c r="C5" s="10">
         <v>5</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="19" t="str">
+      <c r="D5" s="39" t="s">
+        <v>455</v>
+      </c>
+      <c r="E5" s="39" t="s">
+        <v>414</v>
+      </c>
+      <c r="F5" s="39" t="s">
+        <v>456</v>
+      </c>
+      <c r="G5" s="39" t="s">
+        <v>457</v>
+      </c>
+      <c r="H5" s="19">
         <f t="shared" ref="H5:H27" si="0">IF(G5="","",IF(G5="Done",1,IF(G5="In review",0.75,IF(G5="Draft",0.4,0))))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I5" s="6"/>
     </row>
@@ -5301,13 +5532,21 @@
       <c r="C6" s="10">
         <v>15</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="19" t="str">
+      <c r="D6" s="39" t="s">
+        <v>454</v>
+      </c>
+      <c r="E6" s="39" t="s">
+        <v>414</v>
+      </c>
+      <c r="F6" s="39" t="s">
+        <v>458</v>
+      </c>
+      <c r="G6" s="39" t="s">
+        <v>457</v>
+      </c>
+      <c r="H6" s="19">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I6" s="6"/>
     </row>
@@ -5321,10 +5560,10 @@
       <c r="C7" s="10">
         <v>5</v>
       </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="39"/>
       <c r="H7" s="19" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -5341,13 +5580,21 @@
       <c r="C8" s="10">
         <v>5</v>
       </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="19" t="str">
+      <c r="D8" s="39" t="s">
+        <v>454</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>414</v>
+      </c>
+      <c r="F8" s="39" t="s">
+        <v>459</v>
+      </c>
+      <c r="G8" s="39" t="s">
+        <v>457</v>
+      </c>
+      <c r="H8" s="19">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I8" s="6"/>
     </row>
@@ -5581,13 +5828,21 @@
       <c r="C20" s="10">
         <v>5</v>
       </c>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="19" t="str">
+      <c r="D20" s="39" t="s">
+        <v>460</v>
+      </c>
+      <c r="E20" s="39" t="s">
+        <v>414</v>
+      </c>
+      <c r="F20" s="39" t="s">
+        <v>461</v>
+      </c>
+      <c r="G20" s="39" t="s">
+        <v>457</v>
+      </c>
+      <c r="H20" s="19">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I20" s="6"/>
     </row>
@@ -5601,13 +5856,21 @@
       <c r="C21" s="10">
         <v>5</v>
       </c>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="19" t="str">
+      <c r="D21" s="39" t="s">
+        <v>462</v>
+      </c>
+      <c r="E21" s="39" t="s">
+        <v>414</v>
+      </c>
+      <c r="F21" s="39" t="s">
+        <v>463</v>
+      </c>
+      <c r="G21" s="39" t="s">
+        <v>457</v>
+      </c>
+      <c r="H21" s="19">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I21" s="6"/>
     </row>
@@ -5735,9 +5998,9 @@
       <c r="B29" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="C29" s="19" t="str">
+      <c r="C29" s="19">
         <f>IFERROR(AVERAGE(H5:H27),"")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -5746,7 +6009,7 @@
       </c>
       <c r="C30" s="10" t="str">
         <f>COUNTIF(G5:G27,"Done")&amp;" of 23"</f>
-        <v>0 of 23</v>
+        <v>5 of 23</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -5756,7 +6019,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose a value from the list." sqref="G5:G27" xr:uid="{00000000-0002-0000-0500-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose a value from the list." sqref="G7 G9:G19 G22:G27" xr:uid="{00000000-0002-0000-0500-000000000000}">
       <formula1>"Not started,Draft,In review,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5891,7 +6154,9 @@
       <c r="C10" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="D10" s="20"/>
+      <c r="D10" s="48" t="s">
+        <v>457</v>
+      </c>
       <c r="E10" s="21"/>
       <c r="F10" s="22"/>
     </row>
@@ -5987,9 +6252,9 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
     <col min="6" max="6" width="44" customWidth="1"/>
-    <col min="7" max="7" width="34" customWidth="1"/>
+    <col min="7" max="7" width="35.7109375" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="34" customWidth="1"/>
+    <col min="9" max="9" width="38.85546875" customWidth="1"/>
     <col min="10" max="10" width="28" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6039,57 +6304,121 @@
       <c r="A5" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="6"/>
+      <c r="B5" s="39" t="s">
+        <v>478</v>
+      </c>
+      <c r="C5" s="39" t="s">
+        <v>414</v>
+      </c>
+      <c r="D5" s="39" t="s">
+        <v>464</v>
+      </c>
+      <c r="E5" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="39" t="s">
+        <v>465</v>
+      </c>
+      <c r="G5" s="39" t="s">
+        <v>466</v>
+      </c>
+      <c r="H5" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="I5" s="39" t="s">
+        <v>467</v>
+      </c>
+      <c r="J5" s="40"/>
     </row>
     <row r="6" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="6"/>
+      <c r="B6" s="39" t="s">
+        <v>478</v>
+      </c>
+      <c r="C6" s="39" t="s">
+        <v>414</v>
+      </c>
+      <c r="D6" s="39" t="s">
+        <v>464</v>
+      </c>
+      <c r="E6" s="39" t="s">
+        <v>468</v>
+      </c>
+      <c r="F6" s="39" t="s">
+        <v>469</v>
+      </c>
+      <c r="G6" s="39" t="s">
+        <v>470</v>
+      </c>
+      <c r="H6" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="I6" s="39" t="s">
+        <v>470</v>
+      </c>
+      <c r="J6" s="40"/>
     </row>
     <row r="7" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="6"/>
+      <c r="B7" s="39" t="s">
+        <v>438</v>
+      </c>
+      <c r="C7" s="39" t="s">
+        <v>414</v>
+      </c>
+      <c r="D7" s="39" t="s">
+        <v>464</v>
+      </c>
+      <c r="E7" s="39" t="s">
+        <v>471</v>
+      </c>
+      <c r="F7" s="39" t="s">
+        <v>472</v>
+      </c>
+      <c r="G7" s="39" t="s">
+        <v>473</v>
+      </c>
+      <c r="H7" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="I7" s="39" t="s">
+        <v>473</v>
+      </c>
+      <c r="J7" s="40"/>
     </row>
     <row r="8" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
         <v>175</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="6"/>
+      <c r="B8" s="39" t="s">
+        <v>438</v>
+      </c>
+      <c r="C8" s="39" t="s">
+        <v>414</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>474</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>475</v>
+      </c>
+      <c r="F8" s="39" t="s">
+        <v>476</v>
+      </c>
+      <c r="G8" s="39" t="s">
+        <v>477</v>
+      </c>
+      <c r="H8" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="I8" s="39" t="s">
+        <v>477</v>
+      </c>
+      <c r="J8" s="40"/>
     </row>
     <row r="9" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
@@ -6601,7 +6930,7 @@
       </c>
       <c r="F46" s="10">
         <f>COUNTIF(H5:H44,"Kept")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
@@ -6643,11 +6972,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose a value from the list." sqref="D5:D44" xr:uid="{00000000-0002-0000-0700-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose a value from the list." sqref="D9:D44" xr:uid="{00000000-0002-0000-0700-000000000000}">
       <formula1>"GitHub Copilot,ChatGPT,Gemini,Claude,Other"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose a value from the list." sqref="H5:H44" xr:uid="{00000000-0002-0000-0700-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose a value from the list." sqref="H9:H44" xr:uid="{00000000-0002-0000-0700-000001000000}">
       <formula1>"Kept,Changed,Rejected"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6711,13 +7040,27 @@
       </c>
     </row>
     <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
+      <c r="A5" s="37">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="E5" s="37">
+        <v>1</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="G5" s="37" t="s">
+        <v>441</v>
+      </c>
       <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
docs: complete Use Case diagram, sync 8 Q&As, resolve docx placeholders and finalize team workbook
</commit_message>
<xml_diff>
--- a/SE_Lab_QT2_Assignment1_Team_Workbook_Template.xlsx
+++ b/SE_Lab_QT2_Assignment1_Team_Workbook_Template.xlsx
@@ -1259,7 +1259,11 @@
         </is>
       </c>
       <c r="G5" s="47" t="n"/>
-      <c r="H5" s="21" t="n"/>
+      <c r="H5" s="21" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
@@ -1293,7 +1297,11 @@
         </is>
       </c>
       <c r="G6" s="47" t="n"/>
-      <c r="H6" s="21" t="n"/>
+      <c r="H6" s="21" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
@@ -1327,7 +1335,11 @@
         </is>
       </c>
       <c r="G7" s="47" t="n"/>
-      <c r="H7" s="21" t="n"/>
+      <c r="H7" s="21" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
@@ -1361,7 +1373,11 @@
         </is>
       </c>
       <c r="G8" s="47" t="n"/>
-      <c r="H8" s="21" t="n"/>
+      <c r="H8" s="21" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
@@ -1395,7 +1411,11 @@
         </is>
       </c>
       <c r="G9" s="47" t="n"/>
-      <c r="H9" s="21" t="n"/>
+      <c r="H9" s="21" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
@@ -1429,7 +1449,11 @@
         </is>
       </c>
       <c r="G10" s="47" t="n"/>
-      <c r="H10" s="21" t="n"/>
+      <c r="H10" s="21" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="25.5" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
@@ -4187,14 +4211,46 @@
           <t>Q04</t>
         </is>
       </c>
-      <c r="B8" s="43" t="n"/>
-      <c r="C8" s="43" t="n"/>
-      <c r="D8" s="43" t="n"/>
-      <c r="E8" s="43" t="n"/>
-      <c r="F8" s="43" t="n"/>
-      <c r="G8" s="43" t="n"/>
-      <c r="H8" s="43" t="n"/>
-      <c r="I8" s="43" t="n"/>
+      <c r="B8" s="43" t="inlineStr">
+        <is>
+          <t>Business &amp; Fare Rules</t>
+        </is>
+      </c>
+      <c r="C8" s="43" t="inlineStr">
+        <is>
+          <t>The problem statement does not specify if multiple passenger types (Adult, Concession, Off-peak) or bulk ticket quantities can be purchased in a single transaction.</t>
+        </is>
+      </c>
+      <c r="D8" s="43" t="inlineStr">
+        <is>
+          <t>Can a user purchase multiple tickets for different fare classes (Adult, Child, Senior) in one transaction, and what is the maximum ticket limit?</t>
+        </is>
+      </c>
+      <c r="E8" s="43" t="inlineStr">
+        <is>
+          <t>Transit Operations Manager</t>
+        </is>
+      </c>
+      <c r="F8" s="43" t="inlineStr">
+        <is>
+          <t>Yes, passengers can select up to 5 tickets per transaction across Standard Adult, Concession (Child/Senior), and Off-peak categories. Total fare is calculated dynamically as the sum.</t>
+        </is>
+      </c>
+      <c r="G8" s="43" t="inlineStr">
+        <is>
+          <t>Affects UI screen S03 (quantity steppers and fare summary) and database schema (Tickets table with Quantity, UnitPrice, FareCategory).</t>
+        </is>
+      </c>
+      <c r="H8" s="43" t="inlineStr">
+        <is>
+          <t>FR2, DR3</t>
+        </is>
+      </c>
+      <c r="I8" s="43" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
       <c r="J8" s="47" t="n"/>
     </row>
     <row r="9" ht="55.5" customHeight="1">
@@ -4203,14 +4259,46 @@
           <t>Q05</t>
         </is>
       </c>
-      <c r="B9" s="43" t="n"/>
-      <c r="C9" s="43" t="n"/>
-      <c r="D9" s="43" t="n"/>
-      <c r="E9" s="43" t="n"/>
-      <c r="F9" s="43" t="n"/>
-      <c r="G9" s="43" t="n"/>
-      <c r="H9" s="43" t="n"/>
-      <c r="I9" s="43" t="n"/>
+      <c r="B9" s="43" t="inlineStr">
+        <is>
+          <t>Payment &amp; Exception Flow</t>
+        </is>
+      </c>
+      <c r="C9" s="43" t="inlineStr">
+        <is>
+          <t>The problem statement mentions credit card transaction validation, but does not clarify the retry policy when a card is declined.</t>
+        </is>
+      </c>
+      <c r="D9" s="43" t="inlineStr">
+        <is>
+          <t>What is the system policy when a credit card payment is declined, and how many retry attempts are permitted before cancelling?</t>
+        </is>
+      </c>
+      <c r="E9" s="43" t="inlineStr">
+        <is>
+          <t>Payment Gateway Partner / Bank</t>
+        </is>
+      </c>
+      <c r="F9" s="43" t="inlineStr">
+        <is>
+          <t>The TVM displays the specific decline reason (e.g. 'Insufficient funds' or 'Card read error'), retains the user's selected journey details, and allows up to 2 retry attempts or switching to QR/Digital Wallet before returning to the home screen.</t>
+        </is>
+      </c>
+      <c r="G9" s="43" t="inlineStr">
+        <is>
+          <t>Avoids frustrating passengers by not wiping their journey configuration on a single card error. Impacts State Chart (Declined state transition) and UI Screen S05/S07.</t>
+        </is>
+      </c>
+      <c r="H9" s="43" t="inlineStr">
+        <is>
+          <t>FR3, FR5, NFR1</t>
+        </is>
+      </c>
+      <c r="I9" s="43" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
       <c r="J9" s="47" t="n"/>
     </row>
     <row r="10" ht="55.5" customHeight="1">
@@ -4219,14 +4307,46 @@
           <t>Q06</t>
         </is>
       </c>
-      <c r="B10" s="43" t="n"/>
-      <c r="C10" s="43" t="n"/>
-      <c r="D10" s="43" t="n"/>
-      <c r="E10" s="43" t="n"/>
-      <c r="F10" s="43" t="n"/>
-      <c r="G10" s="43" t="n"/>
-      <c r="H10" s="43" t="n"/>
-      <c r="I10" s="43" t="n"/>
+      <c r="B10" s="43" t="inlineStr">
+        <is>
+          <t>Reliability &amp; Architecture</t>
+        </is>
+      </c>
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>The problem statement does not specify how the TVM behaves when internet connectivity to the central server or bank gateway is interrupted.</t>
+        </is>
+      </c>
+      <c r="D10" s="43" t="inlineStr">
+        <is>
+          <t>How should the TVM behave during network disconnections from the central server or payment gateway?</t>
+        </is>
+      </c>
+      <c r="E10" s="43" t="inlineStr">
+        <is>
+          <t>Infrastructure &amp; IT Operations</t>
+        </is>
+      </c>
+      <c r="F10" s="43" t="inlineStr">
+        <is>
+          <t>If central server connection is lost, TVM operates in standalone mode using locally cached station/fare tables and local in-memory transaction buffer; if payment gateway is unreachable, card/QR options show 'Temporarily Unavailable' and notify central monitoring.</t>
+        </is>
+      </c>
+      <c r="G10" s="43" t="inlineStr">
+        <is>
+          <t>Requires local fallback database cache (implemented via in-memory repository in C# demo) and health check monitoring heartbeat.</t>
+        </is>
+      </c>
+      <c r="H10" s="43" t="inlineStr">
+        <is>
+          <t>NFR3, FR8</t>
+        </is>
+      </c>
+      <c r="I10" s="43" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
       <c r="J10" s="47" t="n"/>
     </row>
     <row r="11" ht="55.5" customHeight="1">
@@ -4235,14 +4355,46 @@
           <t>Q07</t>
         </is>
       </c>
-      <c r="B11" s="43" t="n"/>
-      <c r="C11" s="43" t="n"/>
-      <c r="D11" s="43" t="n"/>
-      <c r="E11" s="43" t="n"/>
-      <c r="F11" s="43" t="n"/>
-      <c r="G11" s="43" t="n"/>
-      <c r="H11" s="43" t="n"/>
-      <c r="I11" s="43" t="n"/>
+      <c r="B11" s="43" t="inlineStr">
+        <is>
+          <t>Domain &amp; Security Standards</t>
+        </is>
+      </c>
+      <c r="C11" s="43" t="inlineStr">
+        <is>
+          <t>The problem statement specifies printing a paper ticket with a barcode, but omits barcode encoding standards and fraud prevention safeguards.</t>
+        </is>
+      </c>
+      <c r="D11" s="43" t="inlineStr">
+        <is>
+          <t>What barcode encoding format should be used, and what data payload must be encoded into the barcode to validate transit entry gates?</t>
+        </is>
+      </c>
+      <c r="E11" s="43" t="inlineStr">
+        <is>
+          <t>Turnstile Gate Vendor</t>
+        </is>
+      </c>
+      <c r="F11" s="43" t="inlineStr">
+        <is>
+          <t>Use Code128 / PDF417 or QR code encoding a digitally signed payload containing TicketID, Origin Station, Destination Station, Issue Timestamp, and a SHA-256 HMAC verification hash valid for 2 hours from issuance.</t>
+        </is>
+      </c>
+      <c r="G11" s="43" t="inlineStr">
+        <is>
+          <t>Prevents ticket duplication and counterfeiting. Directly implemented in C# BarcodeRenderer and Ticket output screen (Screen S10).</t>
+        </is>
+      </c>
+      <c r="H11" s="43" t="inlineStr">
+        <is>
+          <t>FR6, DR1, NFR4</t>
+        </is>
+      </c>
+      <c r="I11" s="43" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
       <c r="J11" s="47" t="n"/>
     </row>
     <row r="12" ht="55.5" customHeight="1">
@@ -4251,14 +4403,46 @@
           <t>Q08</t>
         </is>
       </c>
-      <c r="B12" s="43" t="n"/>
-      <c r="C12" s="43" t="n"/>
-      <c r="D12" s="43" t="n"/>
-      <c r="E12" s="43" t="n"/>
-      <c r="F12" s="43" t="n"/>
-      <c r="G12" s="43" t="n"/>
-      <c r="H12" s="43" t="n"/>
-      <c r="I12" s="43" t="n"/>
+      <c r="B12" s="43" t="inlineStr">
+        <is>
+          <t>System Scope &amp; Multi-Line</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="inlineStr">
+        <is>
+          <t>The problem statement refers to selling public transportation tickets (Bus, MRT, etc.) without defining multi-line transfer boundaries.</t>
+        </is>
+      </c>
+      <c r="D12" s="43" t="inlineStr">
+        <is>
+          <t>Does this TVM version support multi-line interchange tickets (e.g. MRT Riverside Line to Central Bus Loop), or is it restricted to single-line journeys?</t>
+        </is>
+      </c>
+      <c r="E12" s="43" t="inlineStr">
+        <is>
+          <t>Transport Authority Project Manager</t>
+        </is>
+      </c>
+      <c r="F12" s="43" t="inlineStr">
+        <is>
+          <t>For Phase 1-4 prototype, the kiosk focuses on the primary MetroLink Riverside Line (7 stations). Transfer routing is reserved for Phase 5 enterprise release.</t>
+        </is>
+      </c>
+      <c r="G12" s="43" t="inlineStr">
+        <is>
+          <t>Keeps prototype scope clearly bounded while demonstrating full end-to-end functionality; architecture designed modularly to support future line plugins.</t>
+        </is>
+      </c>
+      <c r="H12" s="43" t="inlineStr">
+        <is>
+          <t>FR1, DR2</t>
+        </is>
+      </c>
+      <c r="I12" s="43" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
       <c r="J12" s="47" t="n"/>
     </row>
     <row r="13" ht="55.5" customHeight="1">
@@ -5184,10 +5368,26 @@
       <c r="C7" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="D7" s="43" t="n"/>
-      <c r="E7" s="43" t="n"/>
-      <c r="F7" s="43" t="n"/>
-      <c r="G7" s="43" t="n"/>
+      <c r="D7" s="43" t="inlineStr">
+        <is>
+          <t>Draw.io / Matplotlib</t>
+        </is>
+      </c>
+      <c r="E7" s="43" t="inlineStr">
+        <is>
+          <t>524H0057</t>
+        </is>
+      </c>
+      <c r="F7" s="43" t="inlineStr">
+        <is>
+          <t>Section 3.1.1</t>
+        </is>
+      </c>
+      <c r="G7" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H7" s="19">
         <f>IF(G7="","",IF(G7="Done",1,IF(G7="In review",0.75,IF(G7="Draft",0.4,0))))</f>
         <v/>
@@ -5248,10 +5448,26 @@
       <c r="C9" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="43" t="n"/>
-      <c r="E9" s="43" t="n"/>
-      <c r="F9" s="43" t="n"/>
-      <c r="G9" s="43" t="n"/>
+      <c r="D9" s="43" t="inlineStr">
+        <is>
+          <t>Draw.io</t>
+        </is>
+      </c>
+      <c r="E9" s="43" t="inlineStr">
+        <is>
+          <t>524H0069</t>
+        </is>
+      </c>
+      <c r="F9" s="43" t="inlineStr">
+        <is>
+          <t>Section 3.2.1</t>
+        </is>
+      </c>
+      <c r="G9" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H9" s="19">
         <f>IF(G9="","",IF(G9="Done",1,IF(G9="In review",0.75,IF(G9="Draft",0.4,0))))</f>
         <v/>
@@ -5272,10 +5488,26 @@
       <c r="C10" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="D10" s="43" t="n"/>
-      <c r="E10" s="43" t="n"/>
-      <c r="F10" s="43" t="n"/>
-      <c r="G10" s="43" t="n"/>
+      <c r="D10" s="43" t="inlineStr">
+        <is>
+          <t>Draw.io</t>
+        </is>
+      </c>
+      <c r="E10" s="43" t="inlineStr">
+        <is>
+          <t>524H0069</t>
+        </is>
+      </c>
+      <c r="F10" s="43" t="inlineStr">
+        <is>
+          <t>Section 3.2.2</t>
+        </is>
+      </c>
+      <c r="G10" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H10" s="19">
         <f>IF(G10="","",IF(G10="Done",1,IF(G10="In review",0.75,IF(G10="Draft",0.4,0))))</f>
         <v/>
@@ -5296,10 +5528,26 @@
       <c r="C11" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="D11" s="43" t="n"/>
-      <c r="E11" s="43" t="n"/>
-      <c r="F11" s="43" t="n"/>
-      <c r="G11" s="43" t="n"/>
+      <c r="D11" s="43" t="inlineStr">
+        <is>
+          <t>Visual Paradigm</t>
+        </is>
+      </c>
+      <c r="E11" s="43" t="inlineStr">
+        <is>
+          <t>524H0069</t>
+        </is>
+      </c>
+      <c r="F11" s="43" t="inlineStr">
+        <is>
+          <t>Section 3.3.1</t>
+        </is>
+      </c>
+      <c r="G11" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H11" s="19">
         <f>IF(G11="","",IF(G11="Done",1,IF(G11="In review",0.75,IF(G11="Draft",0.4,0))))</f>
         <v/>
@@ -5320,10 +5568,26 @@
       <c r="C12" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="D12" s="43" t="n"/>
-      <c r="E12" s="43" t="n"/>
-      <c r="F12" s="43" t="n"/>
-      <c r="G12" s="43" t="n"/>
+      <c r="D12" s="43" t="inlineStr">
+        <is>
+          <t>Visual Paradigm</t>
+        </is>
+      </c>
+      <c r="E12" s="43" t="inlineStr">
+        <is>
+          <t>524H0069</t>
+        </is>
+      </c>
+      <c r="F12" s="43" t="inlineStr">
+        <is>
+          <t>Section 3.3.2</t>
+        </is>
+      </c>
+      <c r="G12" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H12" s="19">
         <f>IF(G12="","",IF(G12="Done",1,IF(G12="In review",0.75,IF(G12="Draft",0.4,0))))</f>
         <v/>
@@ -5344,10 +5608,26 @@
       <c r="C13" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="D13" s="43" t="n"/>
-      <c r="E13" s="43" t="n"/>
-      <c r="F13" s="43" t="n"/>
-      <c r="G13" s="43" t="n"/>
+      <c r="D13" s="43" t="inlineStr">
+        <is>
+          <t>Visual Studio / Draw.io</t>
+        </is>
+      </c>
+      <c r="E13" s="43" t="inlineStr">
+        <is>
+          <t>524H0069</t>
+        </is>
+      </c>
+      <c r="F13" s="43" t="inlineStr">
+        <is>
+          <t>Section 3.3.3</t>
+        </is>
+      </c>
+      <c r="G13" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H13" s="19">
         <f>IF(G13="","",IF(G13="Done",1,IF(G13="In review",0.75,IF(G13="Draft",0.4,0))))</f>
         <v/>
@@ -5368,10 +5648,26 @@
       <c r="C14" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="D14" s="43" t="n"/>
-      <c r="E14" s="43" t="n"/>
-      <c r="F14" s="43" t="n"/>
-      <c r="G14" s="43" t="n"/>
+      <c r="D14" s="43" t="inlineStr">
+        <is>
+          <t>Figma</t>
+        </is>
+      </c>
+      <c r="E14" s="43" t="inlineStr">
+        <is>
+          <t>524H0069</t>
+        </is>
+      </c>
+      <c r="F14" s="43" t="inlineStr">
+        <is>
+          <t>Section 4.1 &amp; Figma Link</t>
+        </is>
+      </c>
+      <c r="G14" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H14" s="19">
         <f>IF(G14="","",IF(G14="Done",1,IF(G14="In review",0.75,IF(G14="Draft",0.4,0))))</f>
         <v/>
@@ -5392,10 +5688,26 @@
       <c r="C15" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="D15" s="43" t="n"/>
-      <c r="E15" s="43" t="n"/>
-      <c r="F15" s="43" t="n"/>
-      <c r="G15" s="43" t="n"/>
+      <c r="D15" s="43" t="inlineStr">
+        <is>
+          <t>Draw.io</t>
+        </is>
+      </c>
+      <c r="E15" s="43" t="inlineStr">
+        <is>
+          <t>524H0069</t>
+        </is>
+      </c>
+      <c r="F15" s="43" t="inlineStr">
+        <is>
+          <t>Section 4.2.1</t>
+        </is>
+      </c>
+      <c r="G15" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H15" s="19">
         <f>IF(G15="","",IF(G15="Done",1,IF(G15="In review",0.75,IF(G15="Draft",0.4,0))))</f>
         <v/>
@@ -5416,10 +5728,26 @@
       <c r="C16" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="D16" s="43" t="n"/>
-      <c r="E16" s="43" t="n"/>
-      <c r="F16" s="43" t="n"/>
-      <c r="G16" s="43" t="n"/>
+      <c r="D16" s="43" t="inlineStr">
+        <is>
+          <t>Draw.io</t>
+        </is>
+      </c>
+      <c r="E16" s="43" t="inlineStr">
+        <is>
+          <t>524H0069</t>
+        </is>
+      </c>
+      <c r="F16" s="43" t="inlineStr">
+        <is>
+          <t>Section 4.2.2</t>
+        </is>
+      </c>
+      <c r="G16" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H16" s="19">
         <f>IF(G16="","",IF(G16="Done",1,IF(G16="In review",0.75,IF(G16="Draft",0.4,0))))</f>
         <v/>
@@ -5440,10 +5768,26 @@
       <c r="C17" s="45" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="43" t="n"/>
-      <c r="E17" s="43" t="n"/>
-      <c r="F17" s="43" t="n"/>
-      <c r="G17" s="43" t="n"/>
+      <c r="D17" s="43" t="inlineStr">
+        <is>
+          <t>Visual Studio 2022</t>
+        </is>
+      </c>
+      <c r="E17" s="43" t="inlineStr">
+        <is>
+          <t>524H0052</t>
+        </is>
+      </c>
+      <c r="F17" s="43" t="inlineStr">
+        <is>
+          <t>Section 5.1.1</t>
+        </is>
+      </c>
+      <c r="G17" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H17" s="19">
         <f>IF(G17="","",IF(G17="Done",1,IF(G17="In review",0.75,IF(G17="Draft",0.4,0))))</f>
         <v/>
@@ -5464,10 +5808,26 @@
       <c r="C18" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="D18" s="43" t="n"/>
-      <c r="E18" s="43" t="n"/>
-      <c r="F18" s="43" t="n"/>
-      <c r="G18" s="43" t="n"/>
+      <c r="D18" s="43" t="inlineStr">
+        <is>
+          <t>Visual Studio 2022</t>
+        </is>
+      </c>
+      <c r="E18" s="43" t="inlineStr">
+        <is>
+          <t>524H0052</t>
+        </is>
+      </c>
+      <c r="F18" s="43" t="inlineStr">
+        <is>
+          <t>Section 5.1.2</t>
+        </is>
+      </c>
+      <c r="G18" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H18" s="19">
         <f>IF(G18="","",IF(G18="Done",1,IF(G18="In review",0.75,IF(G18="Draft",0.4,0))))</f>
         <v/>
@@ -5488,10 +5848,26 @@
       <c r="C19" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="D19" s="43" t="n"/>
-      <c r="E19" s="43" t="n"/>
-      <c r="F19" s="43" t="n"/>
-      <c r="G19" s="43" t="n"/>
+      <c r="D19" s="43" t="inlineStr">
+        <is>
+          <t>Visual Studio 2022</t>
+        </is>
+      </c>
+      <c r="E19" s="43" t="inlineStr">
+        <is>
+          <t>524H0052</t>
+        </is>
+      </c>
+      <c r="F19" s="43" t="inlineStr">
+        <is>
+          <t>Section 5.1.3</t>
+        </is>
+      </c>
+      <c r="G19" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H19" s="19">
         <f>IF(G19="","",IF(G19="Done",1,IF(G19="In review",0.75,IF(G19="Draft",0.4,0))))</f>
         <v/>
@@ -5592,10 +5968,26 @@
       <c r="C22" s="45" t="n">
         <v>4</v>
       </c>
-      <c r="D22" s="43" t="n"/>
-      <c r="E22" s="43" t="n"/>
-      <c r="F22" s="43" t="n"/>
-      <c r="G22" s="43" t="n"/>
+      <c r="D22" s="43" t="inlineStr">
+        <is>
+          <t>Visual C# WinForms</t>
+        </is>
+      </c>
+      <c r="E22" s="43" t="inlineStr">
+        <is>
+          <t>524H0052</t>
+        </is>
+      </c>
+      <c r="F22" s="43" t="inlineStr">
+        <is>
+          <t>src/SmartTicketing.UI</t>
+        </is>
+      </c>
+      <c r="G22" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H22" s="19">
         <f>IF(G22="","",IF(G22="Done",1,IF(G22="In review",0.75,IF(G22="Draft",0.4,0))))</f>
         <v/>
@@ -5616,10 +6008,26 @@
       <c r="C23" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="D23" s="43" t="n"/>
-      <c r="E23" s="43" t="n"/>
-      <c r="F23" s="43" t="n"/>
-      <c r="G23" s="43" t="n"/>
+      <c r="D23" s="43" t="inlineStr">
+        <is>
+          <t>Visual C# WinForms</t>
+        </is>
+      </c>
+      <c r="E23" s="43" t="inlineStr">
+        <is>
+          <t>524H0052</t>
+        </is>
+      </c>
+      <c r="F23" s="43" t="inlineStr">
+        <is>
+          <t>src/SmartTicketing.UI</t>
+        </is>
+      </c>
+      <c r="G23" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H23" s="19">
         <f>IF(G23="","",IF(G23="Done",1,IF(G23="In review",0.75,IF(G23="Draft",0.4,0))))</f>
         <v/>
@@ -5640,10 +6048,26 @@
       <c r="C24" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="D24" s="43" t="n"/>
-      <c r="E24" s="43" t="n"/>
-      <c r="F24" s="43" t="n"/>
-      <c r="G24" s="43" t="n"/>
+      <c r="D24" s="43" t="inlineStr">
+        <is>
+          <t>MSSQL &amp; T-SQL</t>
+        </is>
+      </c>
+      <c r="E24" s="43" t="inlineStr">
+        <is>
+          <t>524H0052</t>
+        </is>
+      </c>
+      <c r="F24" s="43" t="inlineStr">
+        <is>
+          <t>Database/Script.sql</t>
+        </is>
+      </c>
+      <c r="G24" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H24" s="19">
         <f>IF(G24="","",IF(G24="Done",1,IF(G24="In review",0.75,IF(G24="Draft",0.4,0))))</f>
         <v/>
@@ -5664,10 +6088,26 @@
       <c r="C25" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="43" t="n"/>
-      <c r="E25" s="43" t="n"/>
-      <c r="F25" s="43" t="n"/>
-      <c r="G25" s="43" t="n"/>
+      <c r="D25" s="43" t="inlineStr">
+        <is>
+          <t>Microsoft Word</t>
+        </is>
+      </c>
+      <c r="E25" s="43" t="inlineStr">
+        <is>
+          <t>524H0052</t>
+        </is>
+      </c>
+      <c r="F25" s="43" t="inlineStr">
+        <is>
+          <t>.docx report</t>
+        </is>
+      </c>
+      <c r="G25" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H25" s="19">
         <f>IF(G25="","",IF(G25="Done",1,IF(G25="In review",0.75,IF(G25="Draft",0.4,0))))</f>
         <v/>
@@ -5688,10 +6128,26 @@
       <c r="C26" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="43" t="n"/>
-      <c r="E26" s="43" t="n"/>
-      <c r="F26" s="43" t="n"/>
-      <c r="G26" s="43" t="n"/>
+      <c r="D26" s="43" t="inlineStr">
+        <is>
+          <t>VS Code / Notepad</t>
+        </is>
+      </c>
+      <c r="E26" s="43" t="inlineStr">
+        <is>
+          <t>524H0052</t>
+        </is>
+      </c>
+      <c r="F26" s="43" t="inlineStr">
+        <is>
+          <t>readme.txt</t>
+        </is>
+      </c>
+      <c r="G26" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H26" s="19">
         <f>IF(G26="","",IF(G26="Done",1,IF(G26="In review",0.75,IF(G26="Draft",0.4,0))))</f>
         <v/>
@@ -5712,10 +6168,26 @@
       <c r="C27" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="43" t="n"/>
-      <c r="E27" s="43" t="n"/>
-      <c r="F27" s="43" t="n"/>
-      <c r="G27" s="43" t="n"/>
+      <c r="D27" s="43" t="inlineStr">
+        <is>
+          <t>Excel / Word</t>
+        </is>
+      </c>
+      <c r="E27" s="43" t="inlineStr">
+        <is>
+          <t>524H0052</t>
+        </is>
+      </c>
+      <c r="F27" s="43" t="inlineStr">
+        <is>
+          <t>Section 7 &amp; readme.txt</t>
+        </is>
+      </c>
+      <c r="G27" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="H27" s="19">
         <f>IF(G27="","",IF(G27="Done",1,IF(G27="In review",0.75,IF(G27="Draft",0.4,0))))</f>
         <v/>
@@ -5839,9 +6311,17 @@
           <t>Use case diagram / descriptions</t>
         </is>
       </c>
-      <c r="D5" s="20" t="n"/>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="E5" s="21" t="n"/>
-      <c r="F5" s="22" t="n"/>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>All 5 use cases (UC01-UC05) depicted in Use Case Diagram (Figure 3.1) have fully mapped descriptions with actors, triggers, pre/post-conditions, and alternative/exception flows.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="45" t="n">
@@ -5857,9 +6337,17 @@
           <t>Descriptions / activity</t>
         </is>
       </c>
-      <c r="D6" s="20" t="n"/>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="E6" s="21" t="n"/>
-      <c r="F6" s="22" t="n"/>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>Steps 1 through 10 of UC01 (Start -&gt; Destination -&gt; TicketConfig -&gt; Payment -&gt; Print -&gt; Dispense) map 1:1 to the swimlanes and action nodes of Activity Diagram Figure 3.2.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="45" t="n">
@@ -5875,9 +6363,17 @@
           <t>Sequence / class</t>
         </is>
       </c>
-      <c r="D7" s="20" t="n"/>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="E7" s="21" t="n"/>
-      <c r="F7" s="22" t="n"/>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>Lifelines (:Passenger, :MainForm, :TVMController, :PaymentGateway, :DatabaseService, :TicketPrinter) and messages match Class Diagram Figure 3.6 methods and properties.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="45" t="n">
@@ -5893,9 +6389,17 @@
           <t>State chart / sequence</t>
         </is>
       </c>
-      <c r="D8" s="20" t="n"/>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="E8" s="21" t="n"/>
-      <c r="F8" s="22" t="n"/>
+      <c r="F8" s="22" t="inlineStr">
+        <is>
+          <t>State chart states (Idle, SelectingDestination, ConfiguringTickets, SelectingPayment, ProcessingPayment, Printing, Completed, Declined, Timeout) match Sequence Diagram lifecycles.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="45" t="n">
@@ -5911,9 +6415,17 @@
           <t>Activity / sequence</t>
         </is>
       </c>
-      <c r="D9" s="20" t="n"/>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="E9" s="21" t="n"/>
-      <c r="F9" s="22" t="n"/>
+      <c r="F9" s="22" t="inlineStr">
+        <is>
+          <t>Card authorization and QR generation handshakes in Figure 3.3 match asynchronous request/response callbacks in Figure 3.4 Sequence Diagram.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="45" t="n">
@@ -5935,7 +6447,11 @@
         </is>
       </c>
       <c r="E10" s="21" t="n"/>
-      <c r="F10" s="22" t="n"/>
+      <c r="F10" s="22" t="inlineStr">
+        <is>
+          <t>UC01 references FR1-FR3; UC02 references FR3, FR5, NFR4; UC03 references FR3-FR5, NFR2; UC04 references FR6, DR1; UC05 references FR7. All traced back to Table 4.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="45" t="n">
@@ -5951,9 +6467,17 @@
           <t>Class / code</t>
         </is>
       </c>
-      <c r="D11" s="20" t="n"/>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="E11" s="21" t="n"/>
-      <c r="F11" s="22" t="n"/>
+      <c r="F11" s="22" t="inlineStr">
+        <is>
+          <t>C# namespace SmartTicketing.Domain.Models matches Class Diagram Figure 3.6 attributes, enums, and relationships verified via Forward Engineering and Code Map Figure 5.2.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="45" t="n">
@@ -5969,9 +6493,17 @@
           <t>Wireframes / descriptions</t>
         </is>
       </c>
-      <c r="D12" s="20" t="n"/>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="E12" s="21" t="n"/>
-      <c r="F12" s="22" t="n"/>
+      <c r="F12" s="22" t="inlineStr">
+        <is>
+          <t>Screen S01 (Welcome), S02 (Destination), S03 (Config), S04 (Payment), S05 (Card), S06 (QR), S10 (Ticket) match Figma mockups and main flow steps sequentially.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="45" t="n">
@@ -5987,9 +6519,17 @@
           <t>Architecture / deployment</t>
         </is>
       </c>
-      <c r="D13" s="20" t="n"/>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="E13" s="21" t="n"/>
-      <c r="F13" s="22" t="n"/>
+      <c r="F13" s="22" t="inlineStr">
+        <is>
+          <t>Both Figure 4.2 (Layered MVC) and Figure 4.3 (Deployment Diagram) depict identical hardware interfaces connecting to Local Controller, MSSQL/In-Memory Cache, and Cloud Gateways.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="45" t="n">
@@ -6005,9 +6545,17 @@
           <t>All diagrams</t>
         </is>
       </c>
-      <c r="D14" s="20" t="n"/>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="E14" s="21" t="n"/>
-      <c r="F14" s="22" t="n"/>
+      <c r="F14" s="22" t="inlineStr">
+        <is>
+          <t>All diagrams adhere to ISO/IEC 19505 standard notation: solid arrows with filled heads, open dashed returns, diamond heads for compositions, boolean guards, and clear swimlanes.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D5:E14">

</xml_diff>